<commit_message>
Some refactoring. bcast and device receiving with nrf & 3 byte address.
</commit_message>
<xml_diff>
--- a/hardware/RCKid2-bom.xlsx
+++ b/hardware/RCKid2-bom.xlsx
@@ -4,14 +4,14 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="BOM_RCKid_RCKid_2024-03-09" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="BOM_RCKid_RCKid_2024-06-25" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="581" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="591" uniqueCount="330">
   <si>
     <t>No.</t>
   </si>
@@ -97,7 +97,7 @@
     <t>B+,B-</t>
   </si>
   <si>
-    <t>HDR-TH_1P-V-M_XKB_X4611WV-01I-C28D40</t>
+    <t>hdr-th_1p-v-m_xkb_x4611wv-01i-c28d40</t>
   </si>
   <si>
     <t>4</t>
@@ -316,7 +316,7 @@
     <t>H1</t>
   </si>
   <si>
-    <t>HDR-TH_4P-P2.54-V-M</t>
+    <t>hdr-th_4p-p2.54-v-m</t>
   </si>
   <si>
     <t>XFCN(兴飞)</t>
@@ -352,7 +352,7 @@
     <t>HOME,VOL_DOWN,VOL_UP</t>
   </si>
   <si>
-    <t>KEY-SMD_B3U-3000PM-B</t>
+    <t>key-smd_b3u-3000pm-b</t>
   </si>
   <si>
     <t>OMRON(欧姆龙)</t>
@@ -382,7 +382,7 @@
     <t>J5,J7,J8,USB1</t>
   </si>
   <si>
-    <t>HDR-M-2.54_1X4</t>
+    <t>hdr-m-2.54_1x4</t>
   </si>
   <si>
     <t>C124378</t>
@@ -451,7 +451,7 @@
     <t>AO3400A</t>
   </si>
   <si>
-    <t>Q6</t>
+    <t>Q6,Q9</t>
   </si>
   <si>
     <t>SOT-23-3_L2.9-W1.6-P1.90-LS2.8-BR</t>
@@ -469,7 +469,7 @@
     <t>AO3401A</t>
   </si>
   <si>
-    <t>Q7,Q8</t>
+    <t>Q8</t>
   </si>
   <si>
     <t>SOT-23_L2.9-W1.3-P1.90-LS2.4-BR</t>
@@ -520,7 +520,7 @@
     <t>10kΩ</t>
   </si>
   <si>
-    <t>R48,R52,R53,R54,R55,R56,R67,R73,R74,R76,R83</t>
+    <t>R48,R52,R54,R55,R56,R67,R73,R74,R76,R83</t>
   </si>
   <si>
     <t>0402WGF1002TCE</t>
@@ -535,7 +535,7 @@
     <t>1kΩ</t>
   </si>
   <si>
-    <t>R49</t>
+    <t>R49,R91,R92</t>
   </si>
   <si>
     <t>0402WGF1001TCE</t>
@@ -679,6 +679,21 @@
     <t>39</t>
   </si>
   <si>
+    <t>4.7kΩ</t>
+  </si>
+  <si>
+    <t>R89,R90</t>
+  </si>
+  <si>
+    <t>0402WGF4701TCE</t>
+  </si>
+  <si>
+    <t>C25900</t>
+  </si>
+  <si>
+    <t>40</t>
+  </si>
+  <si>
     <t>DM3CS-SF</t>
   </si>
   <si>
@@ -694,7 +709,7 @@
     <t>C202111</t>
   </si>
   <si>
-    <t>40</t>
+    <t>41</t>
   </si>
   <si>
     <t>SRV05-4-P-T7</t>
@@ -712,7 +727,7 @@
     <t>C85364</t>
   </si>
   <si>
-    <t>41</t>
+    <t>42</t>
   </si>
   <si>
     <t>INA219AIDCNR</t>
@@ -730,7 +745,7 @@
     <t>C87469</t>
   </si>
   <si>
-    <t>42</t>
+    <t>43</t>
   </si>
   <si>
     <t>WMM7040DTHN0-8/TR</t>
@@ -745,7 +760,7 @@
     <t>C9900000758</t>
   </si>
   <si>
-    <t>43</t>
+    <t>44</t>
   </si>
   <si>
     <t>ST7789V 2.8&amp;quot; IPS 320x240 37P 8080 8bit</t>
@@ -757,19 +772,19 @@
     <t>ST7789V 2.8\" IPS DISPLAY 320X240 37P</t>
   </si>
   <si>
-    <t>44</t>
+    <t>45</t>
   </si>
   <si>
     <t>RCKid2 Cartridge Connector Female</t>
   </si>
   <si>
-    <t>U14</t>
-  </si>
-  <si>
-    <t>RCKid Cartridge Riser</t>
-  </si>
-  <si>
-    <t>45</t>
+    <t>U14,U35</t>
+  </si>
+  <si>
+    <t>rckid cartridge riser</t>
+  </si>
+  <si>
+    <t>46</t>
   </si>
   <si>
     <t>SN74LVC2G17DBVR</t>
@@ -784,7 +799,7 @@
     <t>C10429</t>
   </si>
   <si>
-    <t>46</t>
+    <t>47</t>
   </si>
   <si>
     <t>PAM8302AASCR</t>
@@ -802,7 +817,7 @@
     <t>C113367</t>
   </si>
   <si>
-    <t>47</t>
+    <t>48</t>
   </si>
   <si>
     <t>TPS7A2030PDBVR</t>
@@ -817,7 +832,7 @@
     <t>C963429</t>
   </si>
   <si>
-    <t>48</t>
+    <t>49</t>
   </si>
   <si>
     <t>HX4002-MFC</t>
@@ -832,7 +847,7 @@
     <t>C172354</t>
   </si>
   <si>
-    <t>49</t>
+    <t>50</t>
   </si>
   <si>
     <t>BMI160</t>
@@ -850,7 +865,7 @@
     <t>C94021</t>
   </si>
   <si>
-    <t>50</t>
+    <t>51</t>
   </si>
   <si>
     <t>LTR-390UV-01</t>
@@ -868,7 +883,7 @@
     <t>C492374</t>
   </si>
   <si>
-    <t>51</t>
+    <t>52</t>
   </si>
   <si>
     <t>{ManufacturerPart!}</t>
@@ -889,7 +904,7 @@
     <t>C2040</t>
   </si>
   <si>
-    <t>52</t>
+    <t>53</t>
   </si>
   <si>
     <t>ATTINY3217-MFR</t>
@@ -907,7 +922,7 @@
     <t>C617969</t>
   </si>
   <si>
-    <t>53</t>
+    <t>54</t>
   </si>
   <si>
     <t>MCP73832T-2ACI/OT</t>
@@ -922,7 +937,7 @@
     <t>C38066</t>
   </si>
   <si>
-    <t>54</t>
+    <t>55</t>
   </si>
   <si>
     <t>SN74LVC1T45DBVR</t>
@@ -934,7 +949,7 @@
     <t>C7843</t>
   </si>
   <si>
-    <t>55</t>
+    <t>56</t>
   </si>
   <si>
     <t>TPS63001DRCR</t>
@@ -949,7 +964,7 @@
     <t>C28060</t>
   </si>
   <si>
-    <t>56</t>
+    <t>57</t>
   </si>
   <si>
     <t>MC-107DM</t>
@@ -967,7 +982,7 @@
     <t>C2874569</t>
   </si>
   <si>
-    <t>57</t>
+    <t>58</t>
   </si>
   <si>
     <t>12MHz</t>
@@ -1362,7 +1377,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J59"/>
+  <dimension ref="A1:J60"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="10" width="20" customWidth="1"/>
@@ -2173,7 +2188,7 @@
         <v>144</v>
       </c>
       <c r="B26" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="C26" t="s">
         <v>145</v>
@@ -2205,7 +2220,7 @@
         <v>150</v>
       </c>
       <c r="B27" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="C27" t="s">
         <v>151</v>
@@ -2301,7 +2316,7 @@
         <v>167</v>
       </c>
       <c r="B30" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="C30" t="s">
         <v>168</v>
@@ -2333,7 +2348,7 @@
         <v>172</v>
       </c>
       <c r="B31" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="C31" t="s">
         <v>173</v>
@@ -2621,7 +2636,7 @@
         <v>221</v>
       </c>
       <c r="B40" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="C40" t="s">
         <v>222</v>
@@ -2630,19 +2645,19 @@
         <v>223</v>
       </c>
       <c r="E40" t="s">
+        <v>158</v>
+      </c>
+      <c r="F40" t="s">
+        <v>222</v>
+      </c>
+      <c r="G40" t="s">
         <v>224</v>
       </c>
-      <c r="F40" t="s">
-        <v>15</v>
-      </c>
-      <c r="G40" t="s">
-        <v>222</v>
-      </c>
       <c r="H40" t="s">
+        <v>160</v>
+      </c>
+      <c r="I40" t="s">
         <v>225</v>
-      </c>
-      <c r="I40" t="s">
-        <v>226</v>
       </c>
       <c r="J40" t="s">
         <v>18</v>
@@ -2650,31 +2665,31 @@
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B41" t="s">
         <v>10</v>
       </c>
       <c r="C41" t="s">
+        <v>227</v>
+      </c>
+      <c r="D41" t="s">
         <v>228</v>
       </c>
-      <c r="D41" t="s">
+      <c r="E41" t="s">
         <v>229</v>
       </c>
-      <c r="E41" t="s">
+      <c r="F41" t="s">
+        <v>15</v>
+      </c>
+      <c r="G41" t="s">
+        <v>227</v>
+      </c>
+      <c r="H41" t="s">
         <v>230</v>
       </c>
-      <c r="F41" t="s">
-        <v>15</v>
-      </c>
-      <c r="G41" t="s">
-        <v>228</v>
-      </c>
-      <c r="H41" t="s">
+      <c r="I41" t="s">
         <v>231</v>
-      </c>
-      <c r="I41" t="s">
-        <v>232</v>
       </c>
       <c r="J41" t="s">
         <v>18</v>
@@ -2682,31 +2697,31 @@
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B42" t="s">
         <v>10</v>
       </c>
       <c r="C42" t="s">
+        <v>233</v>
+      </c>
+      <c r="D42" t="s">
         <v>234</v>
       </c>
-      <c r="D42" t="s">
+      <c r="E42" t="s">
         <v>235</v>
       </c>
-      <c r="E42" t="s">
+      <c r="F42" t="s">
+        <v>15</v>
+      </c>
+      <c r="G42" t="s">
+        <v>233</v>
+      </c>
+      <c r="H42" t="s">
         <v>236</v>
       </c>
-      <c r="F42" t="s">
-        <v>15</v>
-      </c>
-      <c r="G42" t="s">
-        <v>234</v>
-      </c>
-      <c r="H42" t="s">
+      <c r="I42" t="s">
         <v>237</v>
-      </c>
-      <c r="I42" t="s">
-        <v>238</v>
       </c>
       <c r="J42" t="s">
         <v>18</v>
@@ -2714,28 +2729,28 @@
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B43" t="s">
         <v>10</v>
       </c>
       <c r="C43" t="s">
+        <v>239</v>
+      </c>
+      <c r="D43" t="s">
         <v>240</v>
       </c>
-      <c r="D43" t="s">
+      <c r="E43" t="s">
         <v>241</v>
       </c>
-      <c r="E43" t="s">
+      <c r="F43" t="s">
+        <v>15</v>
+      </c>
+      <c r="G43" t="s">
+        <v>239</v>
+      </c>
+      <c r="H43" t="s">
         <v>242</v>
-      </c>
-      <c r="F43" t="s">
-        <v>15</v>
-      </c>
-      <c r="G43" t="s">
-        <v>240</v>
-      </c>
-      <c r="H43" t="s">
-        <v>15</v>
       </c>
       <c r="I43" t="s">
         <v>243</v>
@@ -2764,33 +2779,33 @@
         <v>15</v>
       </c>
       <c r="G44" t="s">
-        <v>15</v>
+        <v>245</v>
       </c>
       <c r="H44" t="s">
         <v>15</v>
       </c>
       <c r="I44" t="s">
-        <v>15</v>
+        <v>248</v>
       </c>
       <c r="J44" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B45" t="s">
         <v>10</v>
       </c>
       <c r="C45" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D45" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="E45" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="F45" t="s">
         <v>15</v>
@@ -2810,34 +2825,34 @@
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B46" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="C46" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D46" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E46" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="F46" t="s">
         <v>15</v>
       </c>
       <c r="G46" t="s">
-        <v>253</v>
+        <v>15</v>
       </c>
       <c r="H46" t="s">
-        <v>237</v>
+        <v>15</v>
       </c>
       <c r="I46" t="s">
-        <v>256</v>
+        <v>15</v>
       </c>
       <c r="J46" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
@@ -2863,10 +2878,10 @@
         <v>258</v>
       </c>
       <c r="H47" t="s">
+        <v>242</v>
+      </c>
+      <c r="I47" t="s">
         <v>261</v>
-      </c>
-      <c r="I47" t="s">
-        <v>262</v>
       </c>
       <c r="J47" t="s">
         <v>18</v>
@@ -2874,28 +2889,28 @@
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B48" t="s">
         <v>10</v>
       </c>
       <c r="C48" t="s">
+        <v>263</v>
+      </c>
+      <c r="D48" t="s">
         <v>264</v>
       </c>
-      <c r="D48" t="s">
+      <c r="E48" t="s">
         <v>265</v>
       </c>
-      <c r="E48" t="s">
+      <c r="F48" t="s">
+        <v>15</v>
+      </c>
+      <c r="G48" t="s">
+        <v>263</v>
+      </c>
+      <c r="H48" t="s">
         <v>266</v>
-      </c>
-      <c r="F48" t="s">
-        <v>15</v>
-      </c>
-      <c r="G48" t="s">
-        <v>264</v>
-      </c>
-      <c r="H48" t="s">
-        <v>237</v>
       </c>
       <c r="I48" t="s">
         <v>267</v>
@@ -2918,7 +2933,7 @@
         <v>270</v>
       </c>
       <c r="E49" t="s">
-        <v>230</v>
+        <v>271</v>
       </c>
       <c r="F49" t="s">
         <v>15</v>
@@ -2927,7 +2942,7 @@
         <v>269</v>
       </c>
       <c r="H49" t="s">
-        <v>271</v>
+        <v>242</v>
       </c>
       <c r="I49" t="s">
         <v>272</v>
@@ -2950,7 +2965,7 @@
         <v>275</v>
       </c>
       <c r="E50" t="s">
-        <v>276</v>
+        <v>235</v>
       </c>
       <c r="F50" t="s">
         <v>15</v>
@@ -2959,10 +2974,10 @@
         <v>274</v>
       </c>
       <c r="H50" t="s">
+        <v>276</v>
+      </c>
+      <c r="I50" t="s">
         <v>277</v>
-      </c>
-      <c r="I50" t="s">
-        <v>278</v>
       </c>
       <c r="J50" t="s">
         <v>18</v>
@@ -2970,31 +2985,31 @@
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B51" t="s">
         <v>10</v>
       </c>
       <c r="C51" t="s">
+        <v>279</v>
+      </c>
+      <c r="D51" t="s">
         <v>280</v>
       </c>
-      <c r="D51" t="s">
+      <c r="E51" t="s">
         <v>281</v>
       </c>
-      <c r="E51" t="s">
+      <c r="F51" t="s">
+        <v>15</v>
+      </c>
+      <c r="G51" t="s">
+        <v>279</v>
+      </c>
+      <c r="H51" t="s">
         <v>282</v>
       </c>
-      <c r="F51" t="s">
-        <v>15</v>
-      </c>
-      <c r="G51" t="s">
-        <v>280</v>
-      </c>
-      <c r="H51" t="s">
+      <c r="I51" t="s">
         <v>283</v>
-      </c>
-      <c r="I51" t="s">
-        <v>284</v>
       </c>
       <c r="J51" t="s">
         <v>18</v>
@@ -3002,31 +3017,31 @@
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B52" t="s">
         <v>10</v>
       </c>
       <c r="C52" t="s">
+        <v>285</v>
+      </c>
+      <c r="D52" t="s">
         <v>286</v>
       </c>
-      <c r="D52" t="s">
+      <c r="E52" t="s">
         <v>287</v>
       </c>
-      <c r="E52" t="s">
+      <c r="F52" t="s">
+        <v>15</v>
+      </c>
+      <c r="G52" t="s">
+        <v>285</v>
+      </c>
+      <c r="H52" t="s">
         <v>288</v>
       </c>
-      <c r="F52" t="s">
-        <v>15</v>
-      </c>
-      <c r="G52" t="s">
+      <c r="I52" t="s">
         <v>289</v>
-      </c>
-      <c r="H52" t="s">
-        <v>290</v>
-      </c>
-      <c r="I52" t="s">
-        <v>291</v>
       </c>
       <c r="J52" t="s">
         <v>18</v>
@@ -3034,31 +3049,31 @@
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="B53" t="s">
         <v>10</v>
       </c>
       <c r="C53" t="s">
+        <v>291</v>
+      </c>
+      <c r="D53" t="s">
+        <v>292</v>
+      </c>
+      <c r="E53" t="s">
         <v>293</v>
       </c>
-      <c r="D53" t="s">
+      <c r="F53" t="s">
+        <v>15</v>
+      </c>
+      <c r="G53" t="s">
         <v>294</v>
       </c>
-      <c r="E53" t="s">
+      <c r="H53" t="s">
         <v>295</v>
       </c>
-      <c r="F53" t="s">
-        <v>15</v>
-      </c>
-      <c r="G53" t="s">
-        <v>293</v>
-      </c>
-      <c r="H53" t="s">
+      <c r="I53" t="s">
         <v>296</v>
-      </c>
-      <c r="I53" t="s">
-        <v>297</v>
       </c>
       <c r="J53" t="s">
         <v>18</v>
@@ -3066,28 +3081,28 @@
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B54" t="s">
         <v>10</v>
       </c>
       <c r="C54" t="s">
+        <v>298</v>
+      </c>
+      <c r="D54" t="s">
         <v>299</v>
       </c>
-      <c r="D54" t="s">
+      <c r="E54" t="s">
         <v>300</v>
       </c>
-      <c r="E54" t="s">
+      <c r="F54" t="s">
+        <v>15</v>
+      </c>
+      <c r="G54" t="s">
+        <v>298</v>
+      </c>
+      <c r="H54" t="s">
         <v>301</v>
-      </c>
-      <c r="F54" t="s">
-        <v>15</v>
-      </c>
-      <c r="G54" t="s">
-        <v>299</v>
-      </c>
-      <c r="H54" t="s">
-        <v>296</v>
       </c>
       <c r="I54" t="s">
         <v>302</v>
@@ -3110,7 +3125,7 @@
         <v>305</v>
       </c>
       <c r="E55" t="s">
-        <v>230</v>
+        <v>306</v>
       </c>
       <c r="F55" t="s">
         <v>15</v>
@@ -3119,10 +3134,10 @@
         <v>304</v>
       </c>
       <c r="H55" t="s">
-        <v>237</v>
+        <v>301</v>
       </c>
       <c r="I55" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="J55" t="s">
         <v>18</v>
@@ -3130,28 +3145,28 @@
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B56" t="s">
         <v>10</v>
       </c>
       <c r="C56" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="D56" t="s">
+        <v>310</v>
+      </c>
+      <c r="E56" t="s">
+        <v>235</v>
+      </c>
+      <c r="F56" t="s">
+        <v>15</v>
+      </c>
+      <c r="G56" t="s">
         <v>309</v>
       </c>
-      <c r="E56" t="s">
-        <v>310</v>
-      </c>
-      <c r="F56" t="s">
-        <v>15</v>
-      </c>
-      <c r="G56" t="s">
-        <v>308</v>
-      </c>
       <c r="H56" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="I56" t="s">
         <v>311</v>
@@ -3183,10 +3198,10 @@
         <v>313</v>
       </c>
       <c r="H57" t="s">
+        <v>242</v>
+      </c>
+      <c r="I57" t="s">
         <v>316</v>
-      </c>
-      <c r="I57" t="s">
-        <v>317</v>
       </c>
       <c r="J57" t="s">
         <v>18</v>
@@ -3194,38 +3209,70 @@
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B58" t="s">
         <v>10</v>
       </c>
       <c r="C58" t="s">
+        <v>318</v>
+      </c>
+      <c r="D58" t="s">
         <v>319</v>
       </c>
-      <c r="D58" t="s">
+      <c r="E58" t="s">
         <v>320</v>
       </c>
-      <c r="E58" t="s">
+      <c r="F58" t="s">
+        <v>15</v>
+      </c>
+      <c r="G58" t="s">
+        <v>318</v>
+      </c>
+      <c r="H58" t="s">
         <v>321</v>
       </c>
-      <c r="F58" t="s">
-        <v>319</v>
-      </c>
-      <c r="G58" t="s">
+      <c r="I58" t="s">
         <v>322</v>
       </c>
-      <c r="H58" t="s">
+      <c r="J58" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
         <v>323</v>
       </c>
-      <c r="I58" t="s">
+      <c r="B59" t="s">
+        <v>10</v>
+      </c>
+      <c r="C59" t="s">
         <v>324</v>
       </c>
-      <c r="J58" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
+      <c r="D59" t="s">
+        <v>325</v>
+      </c>
+      <c r="E59" t="s">
+        <v>326</v>
+      </c>
+      <c r="F59" t="s">
+        <v>324</v>
+      </c>
+      <c r="G59" t="s">
+        <v>327</v>
+      </c>
+      <c r="H59" t="s">
+        <v>328</v>
+      </c>
+      <c r="I59" t="s">
+        <v>329</v>
+      </c>
+      <c r="J59" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>